<commit_message>
Complete YesBank Collection report generation engine
</commit_message>
<xml_diff>
--- a/templates/YesBank/YesBank_Collection_Template_2026-27.xlsx
+++ b/templates/YesBank/YesBank_Collection_Template_2026-27.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Rachit Goyal\Downloads\audit-report-generator\templates\YesBank\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2AF1C5EA-E1DE-40C9-B84A-A71F92BFCE34}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{18A60D0A-D72C-426E-94E8-AB69134BD80D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{E366AD21-7E7D-48B4-B5AD-0A6D4540711A}"/>
   </bookViews>
@@ -25,7 +25,7 @@
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">Agency!$A$1:$O$69</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Annexure-4'!$A$3:$D$3</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">KAF!$A$1:$AB$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">KAF!$B$1:$AC$1</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -46,7 +46,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="740" uniqueCount="314">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="742" uniqueCount="315">
   <si>
     <t>YES Bank Collection Agency Audit</t>
   </si>
@@ -1080,7 +1080,10 @@
     <t>Yes, Call intensity was followed by the agency as per COC guidelines</t>
   </si>
   <si>
-    <t>KGAC</t>
+    <t>Sr. No</t>
+  </si>
+  <si>
+    <t>Kumar Gaurav Agarwal &amp; Company</t>
   </si>
 </sst>
 </file>
@@ -1093,7 +1096,7 @@
     <numFmt numFmtId="166" formatCode="0_);[Red]\(0\)"/>
     <numFmt numFmtId="167" formatCode="[$-409]d\-mmm\-yy;@"/>
   </numFmts>
-  <fonts count="27" x14ac:knownFonts="1">
+  <fonts count="28" x14ac:knownFonts="1">
     <font>
       <sz val="10"/>
       <name val="Arial"/>
@@ -1261,6 +1264,12 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Cambria"/>
+      <family val="2"/>
+    </font>
   </fonts>
   <fills count="7">
     <fill>
@@ -1299,7 +1308,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="16">
+  <borders count="19">
     <border>
       <left/>
       <right/>
@@ -1516,8 +1525,49 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
-  <cellStyleXfs count="11">
+  <cellStyleXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="5" fillId="3" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
@@ -1529,8 +1579,9 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="27" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="157">
+  <cellXfs count="161">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1961,6 +2012,16 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="16" xfId="4" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment vertical="top"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="6" borderId="17" xfId="11" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="6" borderId="7" xfId="11" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -2011,8 +2072,11 @@
     <xf numFmtId="0" fontId="9" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
   </cellXfs>
-  <cellStyles count="11">
+  <cellStyles count="12">
     <cellStyle name="_Amar's Vehicle_Audit_Report_auto_july_agt_06_Nasik Auto Jan. 07_cv_PIVOT 1_SERIES 2" xfId="7" xr:uid="{80A8BD56-6ED2-42AB-AA86-B312A219BC06}"/>
     <cellStyle name="_Budg based on trend 1_CPC-RPC BSC SEPT-06_Book6_Branch_Metrics_CPA_Final_APR 09  BM UPLOAD_2" xfId="6" xr:uid="{28E173ED-E52B-43E0-9A01-6200B33124B0}"/>
     <cellStyle name="DataPilot Category" xfId="3" xr:uid="{C2EC733E-5CFA-407E-B51E-3AC609C5D00F}"/>
@@ -2020,6 +2084,7 @@
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
     <cellStyle name="Normal 12" xfId="9" xr:uid="{FFDD31A4-3149-42E5-96DD-6A6E1E53F612}"/>
     <cellStyle name="Normal 2" xfId="5" xr:uid="{A6F519D4-B5BB-4C5C-BDDC-95796F400E88}"/>
+    <cellStyle name="Normal 2 3" xfId="11" xr:uid="{F3E4BDBD-6E3C-4888-B20F-65F67C3D77BC}"/>
     <cellStyle name="Normal 3" xfId="10" xr:uid="{42B7EA57-F015-484E-8E89-09920FFF5840}"/>
     <cellStyle name="Normal_DM_1" xfId="4" xr:uid="{47B18B6C-E73C-4527-9963-C930DB66557B}"/>
     <cellStyle name="Normal_Sheet1" xfId="8" xr:uid="{09FDA902-1D9B-48A7-B13B-EDDE10EE22BC}"/>
@@ -2383,14 +2448,14 @@
   <sheetData>
     <row r="1" spans="2:11" ht="14.4" thickBot="1" x14ac:dyDescent="0.35"/>
     <row r="2" spans="2:11" ht="14.4" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B2" s="144" t="s">
+      <c r="B2" s="147" t="s">
         <v>0</v>
       </c>
-      <c r="C2" s="145"/>
-      <c r="D2" s="145"/>
-      <c r="E2" s="145"/>
-      <c r="F2" s="145"/>
-      <c r="G2" s="146"/>
+      <c r="C2" s="148"/>
+      <c r="D2" s="148"/>
+      <c r="E2" s="148"/>
+      <c r="F2" s="148"/>
+      <c r="G2" s="149"/>
     </row>
     <row r="5" spans="2:11" x14ac:dyDescent="0.3">
       <c r="B5" s="2" t="s">
@@ -2430,8 +2495,8 @@
       <c r="F7" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="G7" s="3" t="s">
-        <v>313</v>
+      <c r="G7" s="160" t="s">
+        <v>314</v>
       </c>
     </row>
     <row r="8" spans="2:11" ht="15.9" customHeight="1" x14ac:dyDescent="0.3">
@@ -2459,7 +2524,9 @@
       <c r="D9" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="E9" s="3"/>
+      <c r="E9" s="3" t="s">
+        <v>71</v>
+      </c>
     </row>
     <row r="10" spans="2:11" ht="15.9" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B10" s="2" t="s">
@@ -2508,19 +2575,19 @@
       <c r="K13" s="9"/>
     </row>
     <row r="14" spans="2:11" x14ac:dyDescent="0.3">
-      <c r="B14" s="147" t="s">
+      <c r="B14" s="150" t="s">
         <v>18</v>
       </c>
-      <c r="C14" s="141" t="s">
+      <c r="C14" s="144" t="s">
         <v>19</v>
       </c>
-      <c r="D14" s="141" t="s">
+      <c r="D14" s="144" t="s">
         <v>20</v>
       </c>
-      <c r="E14" s="141" t="s">
+      <c r="E14" s="144" t="s">
         <v>21</v>
       </c>
-      <c r="F14" s="141" t="s">
+      <c r="F14" s="144" t="s">
         <v>22</v>
       </c>
       <c r="G14" s="10"/>
@@ -2530,11 +2597,11 @@
       <c r="K14" s="10"/>
     </row>
     <row r="15" spans="2:11" x14ac:dyDescent="0.3">
-      <c r="B15" s="148"/>
-      <c r="C15" s="142"/>
-      <c r="D15" s="142"/>
-      <c r="E15" s="142"/>
-      <c r="F15" s="142"/>
+      <c r="B15" s="151"/>
+      <c r="C15" s="145"/>
+      <c r="D15" s="145"/>
+      <c r="E15" s="145"/>
+      <c r="F15" s="145"/>
       <c r="G15" s="11"/>
       <c r="H15" s="11"/>
       <c r="I15" s="11"/>
@@ -2642,7 +2709,7 @@
         <f t="shared" si="0"/>
         <v>1</v>
       </c>
-      <c r="F21" s="141" t="str">
+      <c r="F21" s="144" t="str">
         <f>IF(ROUNDUP(E21,2)&lt;60%,"C",IF(ROUNDUP(E21,2)&lt;70%,"C+",IF(ROUNDUP(E21,2)&lt;80%,"B",IF(ROUNDUP(E21,2)&lt;90%,"B+",IF(ROUNDUP(E21,2)&lt;100%,"A","A+")))))</f>
         <v>A+</v>
       </c>
@@ -2651,13 +2718,13 @@
       <c r="B22" s="18" t="s">
         <v>29</v>
       </c>
-      <c r="C22" s="143" t="str">
+      <c r="C22" s="146" t="str">
         <f>VLOOKUP($F$21,$C$27:$D$33,2,FALSE)</f>
         <v>Excellent</v>
       </c>
-      <c r="D22" s="143"/>
-      <c r="E22" s="143"/>
-      <c r="F22" s="142"/>
+      <c r="D22" s="146"/>
+      <c r="E22" s="146"/>
+      <c r="F22" s="145"/>
     </row>
     <row r="26" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B26" s="19" t="s">
@@ -5579,12 +5646,12 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9D599F91-A01D-4D1C-B538-B94856059891}">
   <sheetPr codeName="Sheet3"/>
-  <dimension ref="A1:AB16"/>
+  <dimension ref="A1:AC16"/>
   <sheetFormatPr defaultColWidth="9.109375" defaultRowHeight="13.8" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="18.33203125" style="140" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="9.44140625" style="140" customWidth="1"/>
     <col min="2" max="2" width="27.6640625" style="140" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="10" style="140" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="22.44140625" style="140" customWidth="1"/>
     <col min="4" max="4" width="9.88671875" style="140" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="12.88671875" style="140" bestFit="1" customWidth="1"/>
     <col min="6" max="7" width="30.6640625" style="140" customWidth="1"/>
@@ -5611,94 +5678,97 @@
     <col min="29" max="16384" width="9.109375" style="140"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:28" s="139" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="99" t="s">
+    <row r="1" spans="1:29" s="139" customFormat="1" ht="14.4" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A1" s="141" t="s">
+        <v>313</v>
+      </c>
+      <c r="B1" s="99" t="s">
         <v>219</v>
       </c>
-      <c r="B1" s="99" t="s">
+      <c r="C1" s="99" t="s">
         <v>220</v>
       </c>
-      <c r="C1" s="99" t="s">
+      <c r="D1" s="99" t="s">
         <v>221</v>
       </c>
-      <c r="D1" s="99" t="s">
+      <c r="E1" s="99" t="s">
         <v>222</v>
       </c>
-      <c r="E1" s="99" t="s">
+      <c r="F1" s="99" t="s">
         <v>223</v>
       </c>
-      <c r="F1" s="99" t="s">
+      <c r="G1" s="99" t="s">
         <v>10</v>
       </c>
-      <c r="G1" s="99" t="s">
+      <c r="H1" s="99" t="s">
         <v>224</v>
       </c>
-      <c r="H1" s="99" t="s">
+      <c r="I1" s="99" t="s">
         <v>60</v>
       </c>
-      <c r="I1" s="99" t="s">
+      <c r="J1" s="99" t="s">
         <v>225</v>
       </c>
-      <c r="J1" s="99" t="s">
+      <c r="K1" s="99" t="s">
         <v>226</v>
       </c>
-      <c r="K1" s="99" t="s">
+      <c r="L1" s="99" t="s">
         <v>227</v>
       </c>
-      <c r="L1" s="99" t="s">
+      <c r="M1" s="99" t="s">
         <v>228</v>
       </c>
-      <c r="M1" s="99" t="s">
+      <c r="N1" s="99" t="s">
         <v>229</v>
       </c>
-      <c r="N1" s="99" t="s">
+      <c r="O1" s="99" t="s">
         <v>230</v>
       </c>
-      <c r="O1" s="99" t="s">
+      <c r="P1" s="99" t="s">
         <v>231</v>
       </c>
-      <c r="P1" s="99" t="s">
+      <c r="Q1" s="99" t="s">
         <v>232</v>
       </c>
-      <c r="Q1" s="99" t="s">
+      <c r="R1" s="99" t="s">
         <v>233</v>
       </c>
-      <c r="R1" s="99" t="s">
+      <c r="S1" s="99" t="s">
         <v>234</v>
       </c>
-      <c r="S1" s="99" t="s">
+      <c r="T1" s="99" t="s">
         <v>235</v>
       </c>
-      <c r="T1" s="99" t="s">
+      <c r="U1" s="99" t="s">
         <v>236</v>
       </c>
-      <c r="U1" s="99" t="s">
+      <c r="V1" s="99" t="s">
         <v>237</v>
       </c>
-      <c r="V1" s="99" t="s">
+      <c r="W1" s="99" t="s">
         <v>238</v>
       </c>
-      <c r="W1" s="99" t="s">
+      <c r="X1" s="99" t="s">
         <v>239</v>
       </c>
-      <c r="X1" s="99" t="s">
+      <c r="Y1" s="99" t="s">
         <v>240</v>
       </c>
-      <c r="Y1" s="99" t="s">
+      <c r="Z1" s="99" t="s">
         <v>241</v>
       </c>
-      <c r="Z1" s="99" t="s">
+      <c r="AA1" s="99" t="s">
         <v>242</v>
       </c>
-      <c r="AA1" s="99" t="s">
+      <c r="AB1" s="99" t="s">
         <v>243</v>
       </c>
-      <c r="AB1" s="99" t="s">
+      <c r="AC1" s="99" t="s">
         <v>244</v>
       </c>
     </row>
-    <row r="2" spans="1:28" x14ac:dyDescent="0.25">
-      <c r="A2" s="22"/>
+    <row r="2" spans="1:29" x14ac:dyDescent="0.25">
+      <c r="A2" s="142"/>
       <c r="B2" s="22"/>
       <c r="C2" s="22"/>
       <c r="D2" s="22"/>
@@ -5726,9 +5796,10 @@
       <c r="Z2" s="22"/>
       <c r="AA2" s="22"/>
       <c r="AB2" s="22"/>
-    </row>
-    <row r="3" spans="1:28" x14ac:dyDescent="0.25">
-      <c r="A3" s="22"/>
+      <c r="AC2" s="22"/>
+    </row>
+    <row r="3" spans="1:29" x14ac:dyDescent="0.25">
+      <c r="A3" s="143"/>
       <c r="B3" s="22"/>
       <c r="C3" s="22"/>
       <c r="D3" s="22"/>
@@ -5756,9 +5827,10 @@
       <c r="Z3" s="22"/>
       <c r="AA3" s="22"/>
       <c r="AB3" s="22"/>
-    </row>
-    <row r="4" spans="1:28" x14ac:dyDescent="0.25">
-      <c r="A4" s="22"/>
+      <c r="AC3" s="22"/>
+    </row>
+    <row r="4" spans="1:29" x14ac:dyDescent="0.25">
+      <c r="A4" s="143"/>
       <c r="B4" s="22"/>
       <c r="C4" s="22"/>
       <c r="D4" s="22"/>
@@ -5786,9 +5858,10 @@
       <c r="Z4" s="22"/>
       <c r="AA4" s="22"/>
       <c r="AB4" s="22"/>
-    </row>
-    <row r="5" spans="1:28" x14ac:dyDescent="0.25">
-      <c r="A5" s="22"/>
+      <c r="AC4" s="22"/>
+    </row>
+    <row r="5" spans="1:29" x14ac:dyDescent="0.25">
+      <c r="A5" s="143"/>
       <c r="B5" s="22"/>
       <c r="C5" s="22"/>
       <c r="D5" s="22"/>
@@ -5816,9 +5889,10 @@
       <c r="Z5" s="22"/>
       <c r="AA5" s="22"/>
       <c r="AB5" s="22"/>
-    </row>
-    <row r="6" spans="1:28" x14ac:dyDescent="0.25">
-      <c r="A6" s="22"/>
+      <c r="AC5" s="22"/>
+    </row>
+    <row r="6" spans="1:29" x14ac:dyDescent="0.25">
+      <c r="A6" s="143"/>
       <c r="B6" s="22"/>
       <c r="C6" s="22"/>
       <c r="D6" s="22"/>
@@ -5846,9 +5920,10 @@
       <c r="Z6" s="22"/>
       <c r="AA6" s="22"/>
       <c r="AB6" s="22"/>
-    </row>
-    <row r="7" spans="1:28" x14ac:dyDescent="0.25">
-      <c r="A7" s="22"/>
+      <c r="AC6" s="22"/>
+    </row>
+    <row r="7" spans="1:29" x14ac:dyDescent="0.25">
+      <c r="A7" s="143"/>
       <c r="B7" s="22"/>
       <c r="C7" s="22"/>
       <c r="D7" s="22"/>
@@ -5876,9 +5951,10 @@
       <c r="Z7" s="22"/>
       <c r="AA7" s="22"/>
       <c r="AB7" s="22"/>
-    </row>
-    <row r="8" spans="1:28" x14ac:dyDescent="0.25">
-      <c r="A8" s="22"/>
+      <c r="AC7" s="22"/>
+    </row>
+    <row r="8" spans="1:29" x14ac:dyDescent="0.25">
+      <c r="A8" s="143"/>
       <c r="B8" s="22"/>
       <c r="C8" s="22"/>
       <c r="D8" s="22"/>
@@ -5906,9 +5982,10 @@
       <c r="Z8" s="22"/>
       <c r="AA8" s="22"/>
       <c r="AB8" s="22"/>
-    </row>
-    <row r="9" spans="1:28" x14ac:dyDescent="0.25">
-      <c r="A9" s="22"/>
+      <c r="AC8" s="22"/>
+    </row>
+    <row r="9" spans="1:29" x14ac:dyDescent="0.25">
+      <c r="A9" s="143"/>
       <c r="B9" s="22"/>
       <c r="C9" s="22"/>
       <c r="D9" s="22"/>
@@ -5936,9 +6013,10 @@
       <c r="Z9" s="22"/>
       <c r="AA9" s="22"/>
       <c r="AB9" s="22"/>
-    </row>
-    <row r="10" spans="1:28" x14ac:dyDescent="0.25">
-      <c r="A10" s="22"/>
+      <c r="AC9" s="22"/>
+    </row>
+    <row r="10" spans="1:29" x14ac:dyDescent="0.25">
+      <c r="A10" s="143"/>
       <c r="B10" s="22"/>
       <c r="C10" s="22"/>
       <c r="D10" s="22"/>
@@ -5966,9 +6044,10 @@
       <c r="Z10" s="22"/>
       <c r="AA10" s="22"/>
       <c r="AB10" s="22"/>
-    </row>
-    <row r="11" spans="1:28" x14ac:dyDescent="0.25">
-      <c r="A11" s="22"/>
+      <c r="AC10" s="22"/>
+    </row>
+    <row r="11" spans="1:29" x14ac:dyDescent="0.25">
+      <c r="A11" s="143"/>
       <c r="B11" s="22"/>
       <c r="C11" s="22"/>
       <c r="D11" s="22"/>
@@ -5996,9 +6075,10 @@
       <c r="Z11" s="22"/>
       <c r="AA11" s="22"/>
       <c r="AB11" s="22"/>
-    </row>
-    <row r="12" spans="1:28" x14ac:dyDescent="0.25">
-      <c r="A12" s="22"/>
+      <c r="AC11" s="22"/>
+    </row>
+    <row r="12" spans="1:29" x14ac:dyDescent="0.25">
+      <c r="A12" s="143"/>
       <c r="B12" s="22"/>
       <c r="C12" s="22"/>
       <c r="D12" s="22"/>
@@ -6026,9 +6106,10 @@
       <c r="Z12" s="22"/>
       <c r="AA12" s="22"/>
       <c r="AB12" s="22"/>
-    </row>
-    <row r="13" spans="1:28" x14ac:dyDescent="0.25">
-      <c r="A13" s="22"/>
+      <c r="AC12" s="22"/>
+    </row>
+    <row r="13" spans="1:29" x14ac:dyDescent="0.25">
+      <c r="A13" s="143"/>
       <c r="B13" s="22"/>
       <c r="C13" s="22"/>
       <c r="D13" s="22"/>
@@ -6056,9 +6137,10 @@
       <c r="Z13" s="22"/>
       <c r="AA13" s="22"/>
       <c r="AB13" s="22"/>
-    </row>
-    <row r="14" spans="1:28" x14ac:dyDescent="0.25">
-      <c r="A14" s="22"/>
+      <c r="AC13" s="22"/>
+    </row>
+    <row r="14" spans="1:29" x14ac:dyDescent="0.25">
+      <c r="A14" s="143"/>
       <c r="B14" s="22"/>
       <c r="C14" s="22"/>
       <c r="D14" s="22"/>
@@ -6086,8 +6168,9 @@
       <c r="Z14" s="22"/>
       <c r="AA14" s="22"/>
       <c r="AB14" s="22"/>
-    </row>
-    <row r="15" spans="1:28" x14ac:dyDescent="0.25">
+      <c r="AC14" s="22"/>
+    </row>
+    <row r="15" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A15" s="22"/>
       <c r="B15" s="22"/>
       <c r="C15" s="22"/>
@@ -6116,8 +6199,9 @@
       <c r="Z15" s="22"/>
       <c r="AA15" s="22"/>
       <c r="AB15" s="22"/>
-    </row>
-    <row r="16" spans="1:28" x14ac:dyDescent="0.25">
+      <c r="AC15" s="22"/>
+    </row>
+    <row r="16" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A16" s="22"/>
       <c r="B16" s="22"/>
       <c r="C16" s="22"/>
@@ -6146,6 +6230,7 @@
       <c r="Z16" s="22"/>
       <c r="AA16" s="22"/>
       <c r="AB16" s="22"/>
+      <c r="AC16" s="22"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -6511,21 +6596,21 @@
       <c r="C3" s="105" t="s">
         <v>262</v>
       </c>
-      <c r="D3" s="149" t="s">
+      <c r="D3" s="152" t="s">
         <v>263</v>
       </c>
-      <c r="E3" s="149"/>
-      <c r="F3" s="150"/>
+      <c r="E3" s="152"/>
+      <c r="F3" s="153"/>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A4" s="151" t="s">
+      <c r="A4" s="154" t="s">
         <v>264</v>
       </c>
-      <c r="B4" s="152"/>
-      <c r="C4" s="152"/>
-      <c r="D4" s="152"/>
-      <c r="E4" s="152"/>
-      <c r="F4" s="153"/>
+      <c r="B4" s="155"/>
+      <c r="C4" s="155"/>
+      <c r="D4" s="155"/>
+      <c r="E4" s="155"/>
+      <c r="F4" s="156"/>
     </row>
   </sheetData>
   <mergeCells count="2">
@@ -6631,11 +6716,11 @@
       </c>
     </row>
     <row r="4" spans="1:5" ht="14.4" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A4" s="154"/>
-      <c r="B4" s="155"/>
-      <c r="C4" s="155"/>
-      <c r="D4" s="155"/>
-      <c r="E4" s="156"/>
+      <c r="A4" s="157"/>
+      <c r="B4" s="158"/>
+      <c r="C4" s="158"/>
+      <c r="D4" s="158"/>
+      <c r="E4" s="159"/>
     </row>
   </sheetData>
   <mergeCells count="1">

</xml_diff>

<commit_message>
Add YesBank redirect and latest Tata updates
</commit_message>
<xml_diff>
--- a/templates/YesBank/YesBank_Collection_Template_2026-27.xlsx
+++ b/templates/YesBank/YesBank_Collection_Template_2026-27.xlsx
@@ -2022,6 +2022,9 @@
     <xf numFmtId="0" fontId="16" fillId="6" borderId="7" xfId="11" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -2071,9 +2074,6 @@
     </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
     </xf>
   </cellXfs>
   <cellStyles count="12">
@@ -2448,14 +2448,14 @@
   <sheetData>
     <row r="1" spans="2:11" ht="14.4" thickBot="1" x14ac:dyDescent="0.35"/>
     <row r="2" spans="2:11" ht="14.4" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B2" s="147" t="s">
+      <c r="B2" s="148" t="s">
         <v>0</v>
       </c>
-      <c r="C2" s="148"/>
-      <c r="D2" s="148"/>
-      <c r="E2" s="148"/>
-      <c r="F2" s="148"/>
-      <c r="G2" s="149"/>
+      <c r="C2" s="149"/>
+      <c r="D2" s="149"/>
+      <c r="E2" s="149"/>
+      <c r="F2" s="149"/>
+      <c r="G2" s="150"/>
     </row>
     <row r="5" spans="2:11" x14ac:dyDescent="0.3">
       <c r="B5" s="2" t="s">
@@ -2495,7 +2495,7 @@
       <c r="F7" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="G7" s="160" t="s">
+      <c r="G7" s="144" t="s">
         <v>314</v>
       </c>
     </row>
@@ -2575,19 +2575,19 @@
       <c r="K13" s="9"/>
     </row>
     <row r="14" spans="2:11" x14ac:dyDescent="0.3">
-      <c r="B14" s="150" t="s">
+      <c r="B14" s="151" t="s">
         <v>18</v>
       </c>
-      <c r="C14" s="144" t="s">
+      <c r="C14" s="145" t="s">
         <v>19</v>
       </c>
-      <c r="D14" s="144" t="s">
+      <c r="D14" s="145" t="s">
         <v>20</v>
       </c>
-      <c r="E14" s="144" t="s">
+      <c r="E14" s="145" t="s">
         <v>21</v>
       </c>
-      <c r="F14" s="144" t="s">
+      <c r="F14" s="145" t="s">
         <v>22</v>
       </c>
       <c r="G14" s="10"/>
@@ -2597,11 +2597,11 @@
       <c r="K14" s="10"/>
     </row>
     <row r="15" spans="2:11" x14ac:dyDescent="0.3">
-      <c r="B15" s="151"/>
-      <c r="C15" s="145"/>
-      <c r="D15" s="145"/>
-      <c r="E15" s="145"/>
-      <c r="F15" s="145"/>
+      <c r="B15" s="152"/>
+      <c r="C15" s="146"/>
+      <c r="D15" s="146"/>
+      <c r="E15" s="146"/>
+      <c r="F15" s="146"/>
       <c r="G15" s="11"/>
       <c r="H15" s="11"/>
       <c r="I15" s="11"/>
@@ -2709,7 +2709,7 @@
         <f t="shared" si="0"/>
         <v>1</v>
       </c>
-      <c r="F21" s="144" t="str">
+      <c r="F21" s="145" t="str">
         <f>IF(ROUNDUP(E21,2)&lt;60%,"C",IF(ROUNDUP(E21,2)&lt;70%,"C+",IF(ROUNDUP(E21,2)&lt;80%,"B",IF(ROUNDUP(E21,2)&lt;90%,"B+",IF(ROUNDUP(E21,2)&lt;100%,"A","A+")))))</f>
         <v>A+</v>
       </c>
@@ -2718,13 +2718,13 @@
       <c r="B22" s="18" t="s">
         <v>29</v>
       </c>
-      <c r="C22" s="146" t="str">
+      <c r="C22" s="147" t="str">
         <f>VLOOKUP($F$21,$C$27:$D$33,2,FALSE)</f>
         <v>Excellent</v>
       </c>
-      <c r="D22" s="146"/>
-      <c r="E22" s="146"/>
-      <c r="F22" s="145"/>
+      <c r="D22" s="147"/>
+      <c r="E22" s="147"/>
+      <c r="F22" s="146"/>
     </row>
     <row r="26" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B26" s="19" t="s">
@@ -6596,21 +6596,21 @@
       <c r="C3" s="105" t="s">
         <v>262</v>
       </c>
-      <c r="D3" s="152" t="s">
+      <c r="D3" s="153" t="s">
         <v>263</v>
       </c>
-      <c r="E3" s="152"/>
-      <c r="F3" s="153"/>
+      <c r="E3" s="153"/>
+      <c r="F3" s="154"/>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A4" s="154" t="s">
+      <c r="A4" s="155" t="s">
         <v>264</v>
       </c>
-      <c r="B4" s="155"/>
-      <c r="C4" s="155"/>
-      <c r="D4" s="155"/>
-      <c r="E4" s="155"/>
-      <c r="F4" s="156"/>
+      <c r="B4" s="156"/>
+      <c r="C4" s="156"/>
+      <c r="D4" s="156"/>
+      <c r="E4" s="156"/>
+      <c r="F4" s="157"/>
     </row>
   </sheetData>
   <mergeCells count="2">
@@ -6716,11 +6716,11 @@
       </c>
     </row>
     <row r="4" spans="1:5" ht="14.4" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A4" s="157"/>
-      <c r="B4" s="158"/>
-      <c r="C4" s="158"/>
-      <c r="D4" s="158"/>
-      <c r="E4" s="159"/>
+      <c r="A4" s="158"/>
+      <c r="B4" s="159"/>
+      <c r="C4" s="159"/>
+      <c r="D4" s="159"/>
+      <c r="E4" s="160"/>
     </row>
   </sheetData>
   <mergeCells count="1">

</xml_diff>